<commit_message>
reduce  the token  expiry time
</commit_message>
<xml_diff>
--- a/backend/downloads/Direct_Attainment_Download/Direct_PO_MCA_2026.xlsx
+++ b/backend/downloads/Direct_Attainment_Download/Direct_PO_MCA_2026.xlsx
@@ -11,9 +11,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="24">
-  <si>
-    <t>CA2301 - Unknown Subject</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="300" uniqueCount="38">
+  <si>
+    <t>CA2301 - Data Structures</t>
   </si>
   <si>
     <t>Course</t>
@@ -83,6 +83,48 @@
   </si>
   <si>
     <t>CA2303</t>
+  </si>
+  <si>
+    <t>CA2304 - Computer Networks</t>
+  </si>
+  <si>
+    <t>CA2304</t>
+  </si>
+  <si>
+    <t>CA2305 - Software Engineering</t>
+  </si>
+  <si>
+    <t>CA2305</t>
+  </si>
+  <si>
+    <t>CA2306 - Object-Oriented Programming (OOP)</t>
+  </si>
+  <si>
+    <t>CA2306</t>
+  </si>
+  <si>
+    <t>CA2307 - Web Development</t>
+  </si>
+  <si>
+    <t>CA2307</t>
+  </si>
+  <si>
+    <t>CA2308 - Artificial Intelligence</t>
+  </si>
+  <si>
+    <t>CA2308</t>
+  </si>
+  <si>
+    <t>CA2309 - Machine Learning</t>
+  </si>
+  <si>
+    <t>CA2309</t>
+  </si>
+  <si>
+    <t>CA2310 - Cyber Security</t>
+  </si>
+  <si>
+    <t>CA2310</t>
   </si>
 </sst>
 </file>
@@ -488,7 +530,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:K28"/>
+  <dimension ref="A1:K98"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -1253,14 +1295,1792 @@
         <v>1.08</v>
       </c>
     </row>
+    <row r="31" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B31" s="2"/>
+      <c r="C31" s="2"/>
+      <c r="D31" s="2"/>
+      <c r="E31" s="2"/>
+      <c r="F31" s="2"/>
+      <c r="G31" s="2"/>
+      <c r="H31" s="2"/>
+      <c r="I31" s="2"/>
+      <c r="J31" s="2"/>
+      <c r="K31" s="2"/>
+    </row>
+    <row r="32" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B32" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="C32" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="D32" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="E32" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="F32" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="G32" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="H32" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="I32" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="J32" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="K32" s="4" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A33" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="B33" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C33" s="5">
+        <v>1</v>
+      </c>
+      <c r="D33" s="5">
+        <v>2</v>
+      </c>
+      <c r="E33" s="5">
+        <v>2</v>
+      </c>
+      <c r="F33" s="5">
+        <v>1</v>
+      </c>
+      <c r="G33" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="H33" s="5">
+        <v>2</v>
+      </c>
+      <c r="I33" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="J33" s="5">
+        <v>1</v>
+      </c>
+      <c r="K33" s="5">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A34" s="5"/>
+      <c r="B34" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C34" s="5">
+        <v>0.5</v>
+      </c>
+      <c r="D34" s="5">
+        <v>2</v>
+      </c>
+      <c r="E34" s="5">
+        <v>3</v>
+      </c>
+      <c r="F34" s="5">
+        <v>2</v>
+      </c>
+      <c r="G34" s="5">
+        <v>1</v>
+      </c>
+      <c r="H34" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="I34" s="5">
+        <v>2</v>
+      </c>
+      <c r="J34" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="K34" s="5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A35" s="5"/>
+      <c r="B35" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C35" s="5">
+        <v>0.8</v>
+      </c>
+      <c r="D35" s="5">
+        <v>1</v>
+      </c>
+      <c r="E35" s="5">
+        <v>1</v>
+      </c>
+      <c r="F35" s="5">
+        <v>3</v>
+      </c>
+      <c r="G35" s="5">
+        <v>2</v>
+      </c>
+      <c r="H35" s="5">
+        <v>3</v>
+      </c>
+      <c r="I35" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="J35" s="5">
+        <v>2</v>
+      </c>
+      <c r="K35" s="5" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A36" s="5"/>
+      <c r="B36" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C36" s="5">
+        <v>1.5</v>
+      </c>
+      <c r="D36" s="5">
+        <v>3</v>
+      </c>
+      <c r="E36" s="5">
+        <v>2</v>
+      </c>
+      <c r="F36" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="G36" s="5">
+        <v>3</v>
+      </c>
+      <c r="H36" s="5">
+        <v>1</v>
+      </c>
+      <c r="I36" s="5">
+        <v>2</v>
+      </c>
+      <c r="J36" s="5">
+        <v>3</v>
+      </c>
+      <c r="K36" s="5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A37" s="5"/>
+      <c r="B37" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="C37" s="5">
+        <v>2</v>
+      </c>
+      <c r="D37" s="5">
+        <v>2</v>
+      </c>
+      <c r="E37" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="F37" s="5">
+        <v>2</v>
+      </c>
+      <c r="G37" s="5">
+        <v>1</v>
+      </c>
+      <c r="H37" s="5">
+        <v>2</v>
+      </c>
+      <c r="I37" s="5">
+        <v>3</v>
+      </c>
+      <c r="J37" s="5">
+        <v>1</v>
+      </c>
+      <c r="K37" s="5" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A38" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="B38" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="C38" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D38" s="5">
+        <v>1.23</v>
+      </c>
+      <c r="E38" s="5">
+        <v>0.91</v>
+      </c>
+      <c r="F38" s="5">
+        <v>1.05</v>
+      </c>
+      <c r="G38" s="5">
+        <v>1.23</v>
+      </c>
+      <c r="H38" s="5">
+        <v>1.24</v>
+      </c>
+      <c r="I38" s="5">
+        <v>1.43</v>
+      </c>
+      <c r="J38" s="5">
+        <v>1.3</v>
+      </c>
+      <c r="K38" s="5">
+        <v>1.08</v>
+      </c>
+    </row>
+    <row r="41" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A41" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B41" s="2"/>
+      <c r="C41" s="2"/>
+      <c r="D41" s="2"/>
+      <c r="E41" s="2"/>
+      <c r="F41" s="2"/>
+      <c r="G41" s="2"/>
+      <c r="H41" s="2"/>
+      <c r="I41" s="2"/>
+      <c r="J41" s="2"/>
+      <c r="K41" s="2"/>
+    </row>
+    <row r="42" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A42" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B42" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="C42" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="D42" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="E42" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="F42" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="G42" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="H42" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="I42" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="J42" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="K42" s="4" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="43" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A43" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="B43" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C43" s="5">
+        <v>1</v>
+      </c>
+      <c r="D43" s="5">
+        <v>2</v>
+      </c>
+      <c r="E43" s="5">
+        <v>2</v>
+      </c>
+      <c r="F43" s="5">
+        <v>1</v>
+      </c>
+      <c r="G43" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="H43" s="5">
+        <v>2</v>
+      </c>
+      <c r="I43" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="J43" s="5">
+        <v>1</v>
+      </c>
+      <c r="K43" s="5">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="44" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A44" s="5"/>
+      <c r="B44" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C44" s="5">
+        <v>0.5</v>
+      </c>
+      <c r="D44" s="5">
+        <v>2</v>
+      </c>
+      <c r="E44" s="5">
+        <v>3</v>
+      </c>
+      <c r="F44" s="5">
+        <v>2</v>
+      </c>
+      <c r="G44" s="5">
+        <v>1</v>
+      </c>
+      <c r="H44" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="I44" s="5">
+        <v>2</v>
+      </c>
+      <c r="J44" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="K44" s="5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="45" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A45" s="5"/>
+      <c r="B45" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C45" s="5">
+        <v>0.8</v>
+      </c>
+      <c r="D45" s="5">
+        <v>1</v>
+      </c>
+      <c r="E45" s="5">
+        <v>1</v>
+      </c>
+      <c r="F45" s="5">
+        <v>3</v>
+      </c>
+      <c r="G45" s="5">
+        <v>2</v>
+      </c>
+      <c r="H45" s="5">
+        <v>3</v>
+      </c>
+      <c r="I45" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="J45" s="5">
+        <v>2</v>
+      </c>
+      <c r="K45" s="5" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="46" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A46" s="5"/>
+      <c r="B46" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C46" s="5">
+        <v>1.5</v>
+      </c>
+      <c r="D46" s="5">
+        <v>3</v>
+      </c>
+      <c r="E46" s="5">
+        <v>2</v>
+      </c>
+      <c r="F46" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="G46" s="5">
+        <v>3</v>
+      </c>
+      <c r="H46" s="5">
+        <v>1</v>
+      </c>
+      <c r="I46" s="5">
+        <v>2</v>
+      </c>
+      <c r="J46" s="5">
+        <v>3</v>
+      </c>
+      <c r="K46" s="5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="47" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A47" s="5"/>
+      <c r="B47" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="C47" s="5">
+        <v>2</v>
+      </c>
+      <c r="D47" s="5">
+        <v>2</v>
+      </c>
+      <c r="E47" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="F47" s="5">
+        <v>2</v>
+      </c>
+      <c r="G47" s="5">
+        <v>1</v>
+      </c>
+      <c r="H47" s="5">
+        <v>2</v>
+      </c>
+      <c r="I47" s="5">
+        <v>3</v>
+      </c>
+      <c r="J47" s="5">
+        <v>1</v>
+      </c>
+      <c r="K47" s="5" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="48" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A48" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="B48" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="C48" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D48" s="5">
+        <v>1.23</v>
+      </c>
+      <c r="E48" s="5">
+        <v>0.91</v>
+      </c>
+      <c r="F48" s="5">
+        <v>1.05</v>
+      </c>
+      <c r="G48" s="5">
+        <v>1.23</v>
+      </c>
+      <c r="H48" s="5">
+        <v>1.24</v>
+      </c>
+      <c r="I48" s="5">
+        <v>1.43</v>
+      </c>
+      <c r="J48" s="5">
+        <v>1.3</v>
+      </c>
+      <c r="K48" s="5">
+        <v>1.08</v>
+      </c>
+    </row>
+    <row r="51" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A51" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B51" s="2"/>
+      <c r="C51" s="2"/>
+      <c r="D51" s="2"/>
+      <c r="E51" s="2"/>
+      <c r="F51" s="2"/>
+      <c r="G51" s="2"/>
+      <c r="H51" s="2"/>
+      <c r="I51" s="2"/>
+      <c r="J51" s="2"/>
+      <c r="K51" s="2"/>
+    </row>
+    <row r="52" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A52" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B52" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="C52" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="D52" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="E52" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="F52" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="G52" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="H52" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="I52" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="J52" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="K52" s="4" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="53" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A53" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="B53" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C53" s="5">
+        <v>1</v>
+      </c>
+      <c r="D53" s="5">
+        <v>2</v>
+      </c>
+      <c r="E53" s="5">
+        <v>2</v>
+      </c>
+      <c r="F53" s="5">
+        <v>1</v>
+      </c>
+      <c r="G53" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="H53" s="5">
+        <v>2</v>
+      </c>
+      <c r="I53" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="J53" s="5">
+        <v>1</v>
+      </c>
+      <c r="K53" s="5">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="54" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A54" s="5"/>
+      <c r="B54" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C54" s="5">
+        <v>0.5</v>
+      </c>
+      <c r="D54" s="5">
+        <v>2</v>
+      </c>
+      <c r="E54" s="5">
+        <v>3</v>
+      </c>
+      <c r="F54" s="5">
+        <v>2</v>
+      </c>
+      <c r="G54" s="5">
+        <v>1</v>
+      </c>
+      <c r="H54" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="I54" s="5">
+        <v>2</v>
+      </c>
+      <c r="J54" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="K54" s="5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="55" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A55" s="5"/>
+      <c r="B55" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C55" s="5">
+        <v>0.8</v>
+      </c>
+      <c r="D55" s="5">
+        <v>1</v>
+      </c>
+      <c r="E55" s="5">
+        <v>1</v>
+      </c>
+      <c r="F55" s="5">
+        <v>3</v>
+      </c>
+      <c r="G55" s="5">
+        <v>2</v>
+      </c>
+      <c r="H55" s="5">
+        <v>3</v>
+      </c>
+      <c r="I55" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="J55" s="5">
+        <v>2</v>
+      </c>
+      <c r="K55" s="5" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="56" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A56" s="5"/>
+      <c r="B56" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C56" s="5">
+        <v>1.5</v>
+      </c>
+      <c r="D56" s="5">
+        <v>3</v>
+      </c>
+      <c r="E56" s="5">
+        <v>2</v>
+      </c>
+      <c r="F56" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="G56" s="5">
+        <v>3</v>
+      </c>
+      <c r="H56" s="5">
+        <v>1</v>
+      </c>
+      <c r="I56" s="5">
+        <v>2</v>
+      </c>
+      <c r="J56" s="5">
+        <v>3</v>
+      </c>
+      <c r="K56" s="5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="57" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A57" s="5"/>
+      <c r="B57" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="C57" s="5">
+        <v>2</v>
+      </c>
+      <c r="D57" s="5">
+        <v>2</v>
+      </c>
+      <c r="E57" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="F57" s="5">
+        <v>2</v>
+      </c>
+      <c r="G57" s="5">
+        <v>1</v>
+      </c>
+      <c r="H57" s="5">
+        <v>2</v>
+      </c>
+      <c r="I57" s="5">
+        <v>3</v>
+      </c>
+      <c r="J57" s="5">
+        <v>1</v>
+      </c>
+      <c r="K57" s="5" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="58" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A58" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="B58" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="C58" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D58" s="5">
+        <v>1.23</v>
+      </c>
+      <c r="E58" s="5">
+        <v>0.91</v>
+      </c>
+      <c r="F58" s="5">
+        <v>1.05</v>
+      </c>
+      <c r="G58" s="5">
+        <v>1.23</v>
+      </c>
+      <c r="H58" s="5">
+        <v>1.24</v>
+      </c>
+      <c r="I58" s="5">
+        <v>1.43</v>
+      </c>
+      <c r="J58" s="5">
+        <v>1.3</v>
+      </c>
+      <c r="K58" s="5">
+        <v>1.08</v>
+      </c>
+    </row>
+    <row r="61" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A61" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B61" s="2"/>
+      <c r="C61" s="2"/>
+      <c r="D61" s="2"/>
+      <c r="E61" s="2"/>
+      <c r="F61" s="2"/>
+      <c r="G61" s="2"/>
+      <c r="H61" s="2"/>
+      <c r="I61" s="2"/>
+      <c r="J61" s="2"/>
+      <c r="K61" s="2"/>
+    </row>
+    <row r="62" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A62" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B62" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="C62" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="D62" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="E62" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="F62" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="G62" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="H62" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="I62" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="J62" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="K62" s="4" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="63" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A63" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="B63" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C63" s="5">
+        <v>1</v>
+      </c>
+      <c r="D63" s="5">
+        <v>2</v>
+      </c>
+      <c r="E63" s="5">
+        <v>2</v>
+      </c>
+      <c r="F63" s="5">
+        <v>1</v>
+      </c>
+      <c r="G63" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="H63" s="5">
+        <v>2</v>
+      </c>
+      <c r="I63" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="J63" s="5">
+        <v>1</v>
+      </c>
+      <c r="K63" s="5">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="64" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A64" s="5"/>
+      <c r="B64" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C64" s="5">
+        <v>0.5</v>
+      </c>
+      <c r="D64" s="5">
+        <v>2</v>
+      </c>
+      <c r="E64" s="5">
+        <v>3</v>
+      </c>
+      <c r="F64" s="5">
+        <v>2</v>
+      </c>
+      <c r="G64" s="5">
+        <v>1</v>
+      </c>
+      <c r="H64" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="I64" s="5">
+        <v>2</v>
+      </c>
+      <c r="J64" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="K64" s="5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="65" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A65" s="5"/>
+      <c r="B65" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C65" s="5">
+        <v>0.8</v>
+      </c>
+      <c r="D65" s="5">
+        <v>1</v>
+      </c>
+      <c r="E65" s="5">
+        <v>1</v>
+      </c>
+      <c r="F65" s="5">
+        <v>3</v>
+      </c>
+      <c r="G65" s="5">
+        <v>2</v>
+      </c>
+      <c r="H65" s="5">
+        <v>3</v>
+      </c>
+      <c r="I65" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="J65" s="5">
+        <v>2</v>
+      </c>
+      <c r="K65" s="5" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="66" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A66" s="5"/>
+      <c r="B66" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C66" s="5">
+        <v>1.5</v>
+      </c>
+      <c r="D66" s="5">
+        <v>3</v>
+      </c>
+      <c r="E66" s="5">
+        <v>2</v>
+      </c>
+      <c r="F66" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="G66" s="5">
+        <v>3</v>
+      </c>
+      <c r="H66" s="5">
+        <v>1</v>
+      </c>
+      <c r="I66" s="5">
+        <v>2</v>
+      </c>
+      <c r="J66" s="5">
+        <v>3</v>
+      </c>
+      <c r="K66" s="5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="67" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A67" s="5"/>
+      <c r="B67" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="C67" s="5">
+        <v>2</v>
+      </c>
+      <c r="D67" s="5">
+        <v>2</v>
+      </c>
+      <c r="E67" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="F67" s="5">
+        <v>2</v>
+      </c>
+      <c r="G67" s="5">
+        <v>1</v>
+      </c>
+      <c r="H67" s="5">
+        <v>2</v>
+      </c>
+      <c r="I67" s="5">
+        <v>3</v>
+      </c>
+      <c r="J67" s="5">
+        <v>1</v>
+      </c>
+      <c r="K67" s="5" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="68" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A68" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="B68" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="C68" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D68" s="5">
+        <v>1.23</v>
+      </c>
+      <c r="E68" s="5">
+        <v>0.91</v>
+      </c>
+      <c r="F68" s="5">
+        <v>1.05</v>
+      </c>
+      <c r="G68" s="5">
+        <v>1.23</v>
+      </c>
+      <c r="H68" s="5">
+        <v>1.24</v>
+      </c>
+      <c r="I68" s="5">
+        <v>1.43</v>
+      </c>
+      <c r="J68" s="5">
+        <v>1.3</v>
+      </c>
+      <c r="K68" s="5">
+        <v>1.08</v>
+      </c>
+    </row>
+    <row r="71" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A71" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B71" s="2"/>
+      <c r="C71" s="2"/>
+      <c r="D71" s="2"/>
+      <c r="E71" s="2"/>
+      <c r="F71" s="2"/>
+      <c r="G71" s="2"/>
+      <c r="H71" s="2"/>
+      <c r="I71" s="2"/>
+      <c r="J71" s="2"/>
+      <c r="K71" s="2"/>
+    </row>
+    <row r="72" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A72" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B72" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="C72" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="D72" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="E72" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="F72" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="G72" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="H72" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="I72" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="J72" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="K72" s="4" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="73" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A73" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="B73" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C73" s="5">
+        <v>1</v>
+      </c>
+      <c r="D73" s="5">
+        <v>2</v>
+      </c>
+      <c r="E73" s="5">
+        <v>2</v>
+      </c>
+      <c r="F73" s="5">
+        <v>1</v>
+      </c>
+      <c r="G73" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="H73" s="5">
+        <v>2</v>
+      </c>
+      <c r="I73" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="J73" s="5">
+        <v>1</v>
+      </c>
+      <c r="K73" s="5">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="74" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A74" s="5"/>
+      <c r="B74" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C74" s="5">
+        <v>0.5</v>
+      </c>
+      <c r="D74" s="5">
+        <v>2</v>
+      </c>
+      <c r="E74" s="5">
+        <v>3</v>
+      </c>
+      <c r="F74" s="5">
+        <v>2</v>
+      </c>
+      <c r="G74" s="5">
+        <v>1</v>
+      </c>
+      <c r="H74" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="I74" s="5">
+        <v>2</v>
+      </c>
+      <c r="J74" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="K74" s="5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="75" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A75" s="5"/>
+      <c r="B75" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C75" s="5">
+        <v>0.8</v>
+      </c>
+      <c r="D75" s="5">
+        <v>1</v>
+      </c>
+      <c r="E75" s="5">
+        <v>1</v>
+      </c>
+      <c r="F75" s="5">
+        <v>3</v>
+      </c>
+      <c r="G75" s="5">
+        <v>2</v>
+      </c>
+      <c r="H75" s="5">
+        <v>3</v>
+      </c>
+      <c r="I75" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="J75" s="5">
+        <v>2</v>
+      </c>
+      <c r="K75" s="5" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="76" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A76" s="5"/>
+      <c r="B76" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C76" s="5">
+        <v>1.5</v>
+      </c>
+      <c r="D76" s="5">
+        <v>3</v>
+      </c>
+      <c r="E76" s="5">
+        <v>2</v>
+      </c>
+      <c r="F76" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="G76" s="5">
+        <v>3</v>
+      </c>
+      <c r="H76" s="5">
+        <v>1</v>
+      </c>
+      <c r="I76" s="5">
+        <v>2</v>
+      </c>
+      <c r="J76" s="5">
+        <v>3</v>
+      </c>
+      <c r="K76" s="5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="77" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A77" s="5"/>
+      <c r="B77" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="C77" s="5">
+        <v>2</v>
+      </c>
+      <c r="D77" s="5">
+        <v>2</v>
+      </c>
+      <c r="E77" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="F77" s="5">
+        <v>2</v>
+      </c>
+      <c r="G77" s="5">
+        <v>1</v>
+      </c>
+      <c r="H77" s="5">
+        <v>2</v>
+      </c>
+      <c r="I77" s="5">
+        <v>3</v>
+      </c>
+      <c r="J77" s="5">
+        <v>1</v>
+      </c>
+      <c r="K77" s="5" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="78" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A78" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="B78" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="C78" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D78" s="5">
+        <v>1.23</v>
+      </c>
+      <c r="E78" s="5">
+        <v>0.91</v>
+      </c>
+      <c r="F78" s="5">
+        <v>1.05</v>
+      </c>
+      <c r="G78" s="5">
+        <v>1.23</v>
+      </c>
+      <c r="H78" s="5">
+        <v>1.24</v>
+      </c>
+      <c r="I78" s="5">
+        <v>1.43</v>
+      </c>
+      <c r="J78" s="5">
+        <v>1.3</v>
+      </c>
+      <c r="K78" s="5">
+        <v>1.08</v>
+      </c>
+    </row>
+    <row r="81" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A81" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B81" s="2"/>
+      <c r="C81" s="2"/>
+      <c r="D81" s="2"/>
+      <c r="E81" s="2"/>
+      <c r="F81" s="2"/>
+      <c r="G81" s="2"/>
+      <c r="H81" s="2"/>
+      <c r="I81" s="2"/>
+      <c r="J81" s="2"/>
+      <c r="K81" s="2"/>
+    </row>
+    <row r="82" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A82" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B82" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="C82" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="D82" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="E82" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="F82" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="G82" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="H82" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="I82" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="J82" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="K82" s="4" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="83" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A83" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="B83" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C83" s="5">
+        <v>1</v>
+      </c>
+      <c r="D83" s="5">
+        <v>2</v>
+      </c>
+      <c r="E83" s="5">
+        <v>2</v>
+      </c>
+      <c r="F83" s="5">
+        <v>1</v>
+      </c>
+      <c r="G83" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="H83" s="5">
+        <v>2</v>
+      </c>
+      <c r="I83" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="J83" s="5">
+        <v>1</v>
+      </c>
+      <c r="K83" s="5">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="84" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A84" s="5"/>
+      <c r="B84" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C84" s="5">
+        <v>0.5</v>
+      </c>
+      <c r="D84" s="5">
+        <v>2</v>
+      </c>
+      <c r="E84" s="5">
+        <v>3</v>
+      </c>
+      <c r="F84" s="5">
+        <v>2</v>
+      </c>
+      <c r="G84" s="5">
+        <v>1</v>
+      </c>
+      <c r="H84" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="I84" s="5">
+        <v>2</v>
+      </c>
+      <c r="J84" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="K84" s="5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="85" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A85" s="5"/>
+      <c r="B85" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C85" s="5">
+        <v>0.8</v>
+      </c>
+      <c r="D85" s="5">
+        <v>1</v>
+      </c>
+      <c r="E85" s="5">
+        <v>1</v>
+      </c>
+      <c r="F85" s="5">
+        <v>3</v>
+      </c>
+      <c r="G85" s="5">
+        <v>2</v>
+      </c>
+      <c r="H85" s="5">
+        <v>3</v>
+      </c>
+      <c r="I85" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="J85" s="5">
+        <v>2</v>
+      </c>
+      <c r="K85" s="5" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="86" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A86" s="5"/>
+      <c r="B86" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C86" s="5">
+        <v>1.5</v>
+      </c>
+      <c r="D86" s="5">
+        <v>3</v>
+      </c>
+      <c r="E86" s="5">
+        <v>2</v>
+      </c>
+      <c r="F86" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="G86" s="5">
+        <v>3</v>
+      </c>
+      <c r="H86" s="5">
+        <v>1</v>
+      </c>
+      <c r="I86" s="5">
+        <v>2</v>
+      </c>
+      <c r="J86" s="5">
+        <v>3</v>
+      </c>
+      <c r="K86" s="5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="87" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A87" s="5"/>
+      <c r="B87" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="C87" s="5">
+        <v>2</v>
+      </c>
+      <c r="D87" s="5">
+        <v>2</v>
+      </c>
+      <c r="E87" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="F87" s="5">
+        <v>2</v>
+      </c>
+      <c r="G87" s="5">
+        <v>1</v>
+      </c>
+      <c r="H87" s="5">
+        <v>2</v>
+      </c>
+      <c r="I87" s="5">
+        <v>3</v>
+      </c>
+      <c r="J87" s="5">
+        <v>1</v>
+      </c>
+      <c r="K87" s="5" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="88" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A88" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="B88" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="C88" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D88" s="5">
+        <v>1.23</v>
+      </c>
+      <c r="E88" s="5">
+        <v>0.91</v>
+      </c>
+      <c r="F88" s="5">
+        <v>1.05</v>
+      </c>
+      <c r="G88" s="5">
+        <v>1.23</v>
+      </c>
+      <c r="H88" s="5">
+        <v>1.24</v>
+      </c>
+      <c r="I88" s="5">
+        <v>1.43</v>
+      </c>
+      <c r="J88" s="5">
+        <v>1.3</v>
+      </c>
+      <c r="K88" s="5">
+        <v>1.08</v>
+      </c>
+    </row>
+    <row r="91" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A91" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B91" s="2"/>
+      <c r="C91" s="2"/>
+      <c r="D91" s="2"/>
+      <c r="E91" s="2"/>
+      <c r="F91" s="2"/>
+      <c r="G91" s="2"/>
+      <c r="H91" s="2"/>
+      <c r="I91" s="2"/>
+      <c r="J91" s="2"/>
+      <c r="K91" s="2"/>
+    </row>
+    <row r="92" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A92" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B92" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="C92" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="D92" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="E92" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="F92" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="G92" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="H92" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="I92" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="J92" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="K92" s="4" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="93" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A93" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="B93" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C93" s="5">
+        <v>1</v>
+      </c>
+      <c r="D93" s="5">
+        <v>2</v>
+      </c>
+      <c r="E93" s="5">
+        <v>2</v>
+      </c>
+      <c r="F93" s="5">
+        <v>1</v>
+      </c>
+      <c r="G93" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="H93" s="5">
+        <v>2</v>
+      </c>
+      <c r="I93" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="J93" s="5">
+        <v>1</v>
+      </c>
+      <c r="K93" s="5">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="94" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A94" s="5"/>
+      <c r="B94" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C94" s="5">
+        <v>0.5</v>
+      </c>
+      <c r="D94" s="5">
+        <v>2</v>
+      </c>
+      <c r="E94" s="5">
+        <v>3</v>
+      </c>
+      <c r="F94" s="5">
+        <v>2</v>
+      </c>
+      <c r="G94" s="5">
+        <v>1</v>
+      </c>
+      <c r="H94" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="I94" s="5">
+        <v>2</v>
+      </c>
+      <c r="J94" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="K94" s="5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="95" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A95" s="5"/>
+      <c r="B95" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C95" s="5">
+        <v>0.8</v>
+      </c>
+      <c r="D95" s="5">
+        <v>1</v>
+      </c>
+      <c r="E95" s="5">
+        <v>1</v>
+      </c>
+      <c r="F95" s="5">
+        <v>3</v>
+      </c>
+      <c r="G95" s="5">
+        <v>2</v>
+      </c>
+      <c r="H95" s="5">
+        <v>3</v>
+      </c>
+      <c r="I95" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="J95" s="5">
+        <v>2</v>
+      </c>
+      <c r="K95" s="5" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="96" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A96" s="5"/>
+      <c r="B96" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C96" s="5">
+        <v>1.5</v>
+      </c>
+      <c r="D96" s="5">
+        <v>3</v>
+      </c>
+      <c r="E96" s="5">
+        <v>2</v>
+      </c>
+      <c r="F96" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="G96" s="5">
+        <v>3</v>
+      </c>
+      <c r="H96" s="5">
+        <v>1</v>
+      </c>
+      <c r="I96" s="5">
+        <v>2</v>
+      </c>
+      <c r="J96" s="5">
+        <v>3</v>
+      </c>
+      <c r="K96" s="5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="97" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A97" s="5"/>
+      <c r="B97" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="C97" s="5">
+        <v>2</v>
+      </c>
+      <c r="D97" s="5">
+        <v>2</v>
+      </c>
+      <c r="E97" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="F97" s="5">
+        <v>2</v>
+      </c>
+      <c r="G97" s="5">
+        <v>1</v>
+      </c>
+      <c r="H97" s="5">
+        <v>2</v>
+      </c>
+      <c r="I97" s="5">
+        <v>3</v>
+      </c>
+      <c r="J97" s="5">
+        <v>1</v>
+      </c>
+      <c r="K97" s="5" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="98" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A98" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="B98" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="C98" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D98" s="5">
+        <v>1.23</v>
+      </c>
+      <c r="E98" s="5">
+        <v>0.91</v>
+      </c>
+      <c r="F98" s="5">
+        <v>1.05</v>
+      </c>
+      <c r="G98" s="5">
+        <v>1.23</v>
+      </c>
+      <c r="H98" s="5">
+        <v>1.24</v>
+      </c>
+      <c r="I98" s="5">
+        <v>1.43</v>
+      </c>
+      <c r="J98" s="5">
+        <v>1.3</v>
+      </c>
+      <c r="K98" s="5">
+        <v>1.08</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="20">
     <mergeCell ref="A1:K1"/>
     <mergeCell ref="A3:A7"/>
     <mergeCell ref="A11:K11"/>
     <mergeCell ref="A13:A17"/>
     <mergeCell ref="A21:K21"/>
     <mergeCell ref="A23:A27"/>
+    <mergeCell ref="A31:K31"/>
+    <mergeCell ref="A33:A37"/>
+    <mergeCell ref="A41:K41"/>
+    <mergeCell ref="A43:A47"/>
+    <mergeCell ref="A51:K51"/>
+    <mergeCell ref="A53:A57"/>
+    <mergeCell ref="A61:K61"/>
+    <mergeCell ref="A63:A67"/>
+    <mergeCell ref="A71:K71"/>
+    <mergeCell ref="A73:A77"/>
+    <mergeCell ref="A81:K81"/>
+    <mergeCell ref="A83:A87"/>
+    <mergeCell ref="A91:K91"/>
+    <mergeCell ref="A93:A97"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>